<commit_message>
feat(agc): import room inventory from the accommodation team's own workbook
The team's sheet is multi-tab with a title row and the header row further
down, so the single-sheet template parser rejected every real file. The
parser now scans all sheets, finds the header row, derives the type from
the sheet name or title, skips the "NO. OF ROOMS" counter column, and
drops the gender column entirely — staff assign and check in delegates
manually, so imported rooms stay ungendered.

🤖 Generated with Codebuff
Co-Authored-By: Codebuff <noreply@codebuff.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/agc-room-inventory-integration.xlsx
+++ b/tests/fixtures/agc-room-inventory-integration.xlsx
@@ -4,67 +4,74 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Room inventory" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Hostels without heater" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="WASL" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="GGL" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="EBPV" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="Instructions" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="22">
-  <si>
-    <t>Accommodation location</t>
-  </si>
-  <si>
-    <t>Building / block</t>
-  </si>
-  <si>
-    <t>Room number or apartment name</t>
-  </si>
-  <si>
-    <t>Room capacity (beds/delegates)</t>
-  </si>
-  <si>
-    <t>Gender designation (blank = any)</t>
-  </si>
-  <si>
-    <t>Mighty Fortress Dormitories</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="22">
+  <si>
+    <t>HOSTEL WITHOUT HEATER</t>
+  </si>
+  <si>
+    <t>NO. OF ROOMS</t>
+  </si>
+  <si>
+    <t>ROOM NUMBER</t>
+  </si>
+  <si>
+    <t>CAPACITY</t>
+  </si>
+  <si>
+    <t>101</t>
+  </si>
+  <si>
+    <t>102</t>
+  </si>
+  <si>
+    <t>103</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>Dorm Hall 1</t>
-  </si>
-  <si>
-    <t>Male</t>
-  </si>
-  <si>
-    <t>Hostels Blocks 1–4</t>
-  </si>
-  <si>
-    <t>Block 1</t>
+    <t>WISE AS SERPENTS</t>
+  </si>
+  <si>
+    <t>ADDITONAL INFORMATION</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>HAS FRIDGE</t>
+  </si>
+  <si>
+    <t>GOOD GENERAL</t>
+  </si>
+  <si>
+    <t>Capacity</t>
   </si>
   <si>
     <t>Room 101</t>
   </si>
   <si>
-    <t>Female</t>
-  </si>
-  <si>
-    <t>Wise as Serpents Lodge</t>
-  </si>
-  <si>
-    <t>WSL Room 1</t>
-  </si>
-  <si>
-    <t>Good General Lodge</t>
-  </si>
-  <si>
-    <t>GGL Room 1</t>
-  </si>
-  <si>
-    <t>Everything by Prayer Village</t>
+    <t>EVERYTHING BY PRAYER VILLAGE</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Apartment name</t>
   </si>
   <si>
     <t>Apartment 1</t>
@@ -73,26 +80,20 @@
     <t>Apartment 2</t>
   </si>
   <si>
-    <t>Not A Real Location</t>
-  </si>
-  <si>
-    <t>Room X</t>
+    <t>One sheet per accommodation type. Keep the title and header rows, then add one room per row. NO. OF ROOMS is only a count and is ignored.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
       <scheme val="minor"/>
       <sz val="11"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
     </font>
   </fonts>
   <fills count="2">
@@ -115,9 +116,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -457,150 +457,294 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="20" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="C3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2">
-        <v>2</v>
-      </c>
-      <c r="E2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>15</v>
+      <c r="C4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>3</v>
       </c>
       <c r="B5" t="s">
         <v>6</v>
       </c>
       <c r="C5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>2</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>16</v>
       </c>
-      <c r="D5">
+      <c r="B1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
         <v>1</v>
       </c>
-      <c r="E5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" t="s">
-        <v>18</v>
-      </c>
-      <c r="D6">
+      <c r="B4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4">
         <v>4</v>
       </c>
-      <c r="E6" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" t="s">
-        <v>19</v>
-      </c>
-      <c r="D7">
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5">
         <v>5</v>
       </c>
-      <c r="E7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" t="s">
-        <v>6</v>
-      </c>
-      <c r="C8" t="s">
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>21</v>
-      </c>
-      <c r="D8">
-        <v>1</v>
-      </c>
-      <c r="E8" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>